<commit_message>
add result eval + plots
</commit_message>
<xml_diff>
--- a/pipeline_eval/eval_results/overall_metrics_report.xlsx
+++ b/pipeline_eval/eval_results/overall_metrics_report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -424,10 +424,20 @@
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
-    <col width="31" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="29" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="31" customWidth="1" min="13" max="13"/>
+    <col width="31" customWidth="1" min="14" max="14"/>
+    <col width="31" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
+    <col width="29" customWidth="1" min="18" max="18"/>
+    <col width="29" customWidth="1" min="19" max="19"/>
+    <col width="29" customWidth="1" min="20" max="20"/>
+    <col width="29" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,78 +458,158 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Micro-Average BM25 Hit Rate@1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Micro-Average BM25 Hit Rate@3</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Micro-Average BM25 Hit Rate@5</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Micro-Average LLM Accuracy</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Micro-Average Cat1 Accuracy</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Micro-Average Cat2 Accuracy</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Micro-Average Cat3 Accuracy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Micro-Average Cat4 Accuracy</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Micro-Average Cat5 Accuracy</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Macro-Average BM25 Hit Rate@1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Macro-Average BM25 Hit Rate@3</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Macro-Average BM25 Hit Rate@5</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Macro-Average LLM Accuracy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Micro-Average BM25 Hit Rate@1</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Micro-Average BM25 Hit Rate@3</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Micro-Average BM25 Hit Rate@5</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Micro-Average LLM Accuracy</t>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Macro-Average Cat1 Accuracy</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Macro-Average Cat2 Accuracy</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Macro-Average Cat3 Accuracy</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Macro-Average Cat4 Accuracy</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Macro-Average Cat5 Accuracy</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B2" t="n">
-        <v>304</v>
+        <v>1683</v>
       </c>
       <c r="C2" t="n">
-        <v>188</v>
+        <v>1036</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6852</v>
+        <v>0.65068330362448</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8282499999999999</v>
+        <v>0.8093285799168152</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8895500000000001</v>
+        <v>0.8685086155674391</v>
       </c>
       <c r="G2" t="n">
-        <v>0.65455</v>
+        <v>0.6155674390968509</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6779605263157895</v>
+        <v>0.6388888888888888</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8263157894736842</v>
+        <v>0.6801346801346801</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8838815789473684</v>
+        <v>0.5280898876404494</v>
       </c>
       <c r="K2" t="n">
-        <v>0.618421052631579</v>
+        <v>0.671919770773639</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.4524495677233429</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.6503777777777777</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.8096777777777777</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.8681222222222222</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.6314666666666666</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.6464717099797745</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.6971558985856371</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.4678710178710179</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.6929787589578192</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.4062208799284275</v>
       </c>
     </row>
   </sheetData>
@@ -533,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -547,6 +637,11 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +700,31 @@
           <t>LLM Judge Accuracy</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Cat1 Accuracy</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Cat2 Accuracy</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Cat3 Accuracy</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Cat4 Accuracy</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Cat5 Accuracy</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -642,6 +762,21 @@
       <c r="K2" t="n">
         <v>0.5377</v>
       </c>
+      <c r="L2" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.8108108108108109</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.6857142857142857</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.1063829787234043</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -678,6 +813,385 @@
       </c>
       <c r="K3" t="n">
         <v>0.7714</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eval_conv_2.xlsx</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>193</v>
+      </c>
+      <c r="D4" t="n">
+        <v>126.6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>155.8</v>
+      </c>
+      <c r="F4" t="n">
+        <v>169.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>131</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.6559</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.8074</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.8778</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.6788</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6129032258064516</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.7790697674418605</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.4634146341463415</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>eval_conv_3.xlsx</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>260</v>
+      </c>
+      <c r="D5" t="n">
+        <v>168.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>205.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>221.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>173</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.6494</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.7904</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.8532999999999999</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.6654</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.7297297297297297</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.5454545454545454</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.7117117117117117</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.459016393442623</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>eval_conv_4.xlsx</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>97</v>
+      </c>
+      <c r="D6" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>72</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.5714</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.7809</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.7423</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.6774193548387096</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.8076923076923077</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>eval_conv_6.xlsx</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>190</v>
+      </c>
+      <c r="D7" t="n">
+        <v>144.7</v>
+      </c>
+      <c r="E7" t="n">
+        <v>172.4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>181</v>
+      </c>
+      <c r="G7" t="n">
+        <v>105</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.7614</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9072</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9528</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.5526</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.4117647058823529</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.5783132530120482</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.575</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>eval_conv_7.xlsx</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>239</v>
+      </c>
+      <c r="D8" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>198</v>
+      </c>
+      <c r="F8" t="n">
+        <v>213.8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>121</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.6282</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.8284</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.8946</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.5063</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.559322033898305</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>eval_conv_8.xlsx</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>196</v>
+      </c>
+      <c r="D9" t="n">
+        <v>117.3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>144.7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>158.7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>114</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.5986</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.7381</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.8099</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.5816</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.5945945945945946</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.4615384615384616</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.6301369863013698</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>eval_conv_9.xlsx</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>204</v>
+      </c>
+      <c r="D10" t="n">
+        <v>126.1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>158.8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>168.9</v>
+      </c>
+      <c r="G10" t="n">
+        <v>132</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.6181</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.7782</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.6471</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.65625</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.6521739130434783</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final: complete eval + img
</commit_message>
<xml_diff>
--- a/pipeline_eval/eval_results/overall_metrics_report.xlsx
+++ b/pipeline_eval/eval_results/overall_metrics_report.xlsx
@@ -416,29 +416,6 @@
   </sheetPr>
   <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="29" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
-    <col width="29" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
-    <col width="29" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
-    <col width="31" customWidth="1" min="14" max="14"/>
-    <col width="31" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="29" customWidth="1" min="17" max="17"/>
-    <col width="29" customWidth="1" min="18" max="18"/>
-    <col width="29" customWidth="1" min="19" max="19"/>
-    <col width="29" customWidth="1" min="20" max="20"/>
-    <col width="29" customWidth="1" min="21" max="21"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -549,67 +526,67 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>1683</v>
+        <v>1986</v>
       </c>
       <c r="C2" t="n">
-        <v>1036</v>
+        <v>1217</v>
       </c>
       <c r="D2" t="n">
-        <v>0.65068330362448</v>
+        <v>0.6581</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8093285799168152</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8685086155674391</v>
+        <v>0.8738</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6155674390968509</v>
+        <v>0.8259</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6388888888888888</v>
+        <v>0.9157</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6801346801346801</v>
+        <v>0.8501</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5280898876404494</v>
+        <v>0.7874</v>
       </c>
       <c r="K2" t="n">
-        <v>0.671919770773639</v>
+        <v>0.8464</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4524495677233429</v>
+        <v>0.6975</v>
       </c>
       <c r="M2" t="n">
-        <v>0.6503777777777777</v>
+        <v>0.6578816515609266</v>
       </c>
       <c r="N2" t="n">
-        <v>0.8096777777777777</v>
+        <v>0.8129392648539777</v>
       </c>
       <c r="O2" t="n">
-        <v>0.8681222222222222</v>
+        <v>0.8740348640483384</v>
       </c>
       <c r="P2" t="n">
-        <v>0.6314666666666666</v>
+        <v>0.8350272507552872</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6464717099797745</v>
+        <v>0.914799834369304</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6971558985856371</v>
+        <v>0.8571398652907163</v>
       </c>
       <c r="S2" t="n">
-        <v>0.4678710178710179</v>
+        <v>0.7679796629571303</v>
       </c>
       <c r="T2" t="n">
-        <v>0.6929787589578192</v>
+        <v>0.8551767221333794</v>
       </c>
       <c r="U2" t="n">
-        <v>0.4062208799284275</v>
+        <v>0.702768931556857</v>
       </c>
     </row>
   </sheetData>
@@ -623,26 +600,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -748,34 +707,34 @@
         <v>173.5</v>
       </c>
       <c r="G2" t="n">
-        <v>107</v>
+        <v>149</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6625</v>
+        <v>0.6624716515609266</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8216</v>
+        <v>0.8216592648539778</v>
       </c>
       <c r="J2" t="n">
-        <v>0.872</v>
+        <v>0.8719448640483384</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5377</v>
+        <v>0.750807250755287</v>
       </c>
       <c r="L2" t="n">
-        <v>0.59375</v>
+        <v>0.8742913960566604</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8108108108108109</v>
+        <v>0.9753391026692105</v>
       </c>
       <c r="N2" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.686710342932177</v>
       </c>
       <c r="O2" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.8451153217894078</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1063829787234043</v>
+        <v>0.371276332630391</v>
       </c>
     </row>
     <row r="3">
@@ -800,34 +759,34 @@
         <v>95.2</v>
       </c>
       <c r="G3" t="n">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7079</v>
+        <v>0.7078716515609266</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8349</v>
+        <v>0.8349592648539778</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9071</v>
+        <v>0.9070448640483384</v>
       </c>
       <c r="K3" t="n">
-        <v>0.7714</v>
+        <v>0.984507250755287</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8181818181818182</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9230769230769231</v>
+        <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>0.3020949583167923</v>
       </c>
       <c r="O3" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.9775828542569404</v>
       </c>
       <c r="P3" t="n">
-        <v>0.5</v>
+        <v>0.7648933539069867</v>
       </c>
     </row>
     <row r="4">
@@ -852,34 +811,34 @@
         <v>169.4</v>
       </c>
       <c r="G4" t="n">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6559</v>
+        <v>0.6558716515609266</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8074</v>
+        <v>0.8074592648539778</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8778</v>
+        <v>0.8777448640483384</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6788</v>
+        <v>0.891907250755287</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.893444621863112</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.9052690325991404</v>
       </c>
       <c r="N4" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7790697674418605</v>
+        <v>0.9384708035169826</v>
       </c>
       <c r="P4" t="n">
-        <v>0.4634146341463415</v>
+        <v>0.7283079880533282</v>
       </c>
     </row>
     <row r="5">
@@ -901,37 +860,37 @@
         <v>205.5</v>
       </c>
       <c r="F5" t="n">
-        <v>221.9</v>
+        <v>221.8</v>
       </c>
       <c r="G5" t="n">
-        <v>173</v>
+        <v>228</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6494</v>
+        <v>0.6493716515609266</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7904</v>
+        <v>0.7904592648539778</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.8532448640483383</v>
       </c>
       <c r="K5" t="n">
-        <v>0.6654</v>
+        <v>0.878507250755287</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7297297297297297</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>0.825</v>
+        <v>0.9895282918583996</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.8475495037713379</v>
       </c>
       <c r="O5" t="n">
-        <v>0.7117117117117117</v>
+        <v>0.8711127477868338</v>
       </c>
       <c r="P5" t="n">
-        <v>0.459016393442623</v>
+        <v>0.7239097473496097</v>
       </c>
     </row>
     <row r="6">
@@ -944,254 +903,306 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>97</v>
+        <v>242</v>
       </c>
       <c r="D6" t="n">
-        <v>55.4</v>
+        <v>179.4</v>
       </c>
       <c r="E6" t="n">
-        <v>75.7</v>
+        <v>212.8</v>
       </c>
       <c r="F6" t="n">
-        <v>79.3</v>
+        <v>222.3</v>
       </c>
       <c r="G6" t="n">
-        <v>72</v>
+        <v>199</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5714</v>
+        <v>0.7413716515609265</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7809</v>
+        <v>0.8791592648539778</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8176</v>
+        <v>0.9185448640483383</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7423</v>
+        <v>0.8205072507552871</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6774193548387096</v>
+        <v>0.95796075089537</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8461538461538461</v>
+        <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.8735235297453638</v>
       </c>
       <c r="O6" t="n">
-        <v>0.8076923076923077</v>
+        <v>0.8977187930844679</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>0.5305183539069867</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>eval_conv_6.xlsx</t>
+          <t>eval_conv_5.xlsx</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>190</v>
+        <v>158</v>
       </c>
       <c r="D7" t="n">
-        <v>144.7</v>
+        <v>87.8</v>
       </c>
       <c r="E7" t="n">
-        <v>172.4</v>
+        <v>117.5</v>
       </c>
       <c r="F7" t="n">
-        <v>181</v>
+        <v>130.6</v>
       </c>
       <c r="G7" t="n">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7614</v>
+        <v>0.5556716515609266</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9072</v>
+        <v>0.7435592648539778</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9528</v>
+        <v>0.8267448640483384</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5526</v>
+        <v>0.8840072507552871</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5</v>
+        <v>0.9138747293899937</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.9145282918583997</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.8735235297453638</v>
       </c>
       <c r="O7" t="n">
-        <v>0.5783132530120482</v>
+        <v>0.9497236167202834</v>
       </c>
       <c r="P7" t="n">
-        <v>0.575</v>
+        <v>0.7220362110498437</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>eval_conv_7.xlsx</t>
+          <t>eval_conv_6.xlsx</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>239</v>
+        <v>190</v>
       </c>
       <c r="D8" t="n">
-        <v>150.1</v>
+        <v>144.7</v>
       </c>
       <c r="E8" t="n">
-        <v>198</v>
+        <v>172.4</v>
       </c>
       <c r="F8" t="n">
-        <v>213.8</v>
+        <v>181</v>
       </c>
       <c r="G8" t="n">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6282</v>
+        <v>0.7613716515609266</v>
       </c>
       <c r="I8" t="n">
-        <v>0.8284</v>
+        <v>0.9072592648539778</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8946</v>
+        <v>0.9527448640483384</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5063</v>
+        <v>0.765707250755287</v>
       </c>
       <c r="L8" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7805413960566604</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5762929977407526</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="O8" t="n">
-        <v>0.559322033898305</v>
+        <v>0.7377142890871703</v>
       </c>
       <c r="P8" t="n">
-        <v>0.5</v>
+        <v>0.8398933539069866</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>eval_conv_8.xlsx</t>
+          <t>eval_conv_7.xlsx</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>196</v>
+        <v>239</v>
       </c>
       <c r="D9" t="n">
-        <v>117.3</v>
+        <v>150.1</v>
       </c>
       <c r="E9" t="n">
-        <v>144.7</v>
+        <v>198</v>
       </c>
       <c r="F9" t="n">
-        <v>158.7</v>
+        <v>213.8</v>
       </c>
       <c r="G9" t="n">
-        <v>114</v>
+        <v>172</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5986</v>
+        <v>0.6281716515609266</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7381</v>
+        <v>0.8284592648539778</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8099</v>
+        <v>0.8945448640483383</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5816</v>
+        <v>0.719407250755287</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5945945945945946</v>
+        <v>0.947208062723327</v>
       </c>
       <c r="M9" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.497861625191733</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4615384615384616</v>
+        <v>0.6020949583167924</v>
       </c>
       <c r="O9" t="n">
-        <v>0.6301369863013698</v>
+        <v>0.7187230699734272</v>
       </c>
       <c r="P9" t="n">
-        <v>0.4</v>
+        <v>0.7648933539069867</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>eval_conv_8.xlsx</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>196</v>
+      </c>
+      <c r="D10" t="n">
+        <v>117.3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>144.7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>158.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>156</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.5985716515609266</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.7381592648539778</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.8098448640483383</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.794707250755287</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.875135990651255</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.891801019131127</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.763633419855254</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.789538022376492</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.6648933539069868</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>eval_conv_9.xlsx</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C11" t="n">
         <v>204</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>126.1</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E11" t="n">
         <v>158.8</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F11" t="n">
         <v>168.9</v>
       </c>
-      <c r="G10" t="n">
-        <v>132</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.6181</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.7782</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.828</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.6471</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.65625</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.6521739130434783</v>
+      <c r="G11" t="n">
+        <v>175</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.6180716515609266</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.7782592648539778</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.8279448640483383</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.860207250755287</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.9055413960566604</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.8207782918583997</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.7306663868882208</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.8260677027417888</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.9170672669504649</v>
       </c>
     </row>
   </sheetData>

</xml_diff>